<commit_message>
Bootstrap punctuation alignment so reordered marks are counted
mine_punct aligned each line's punctuation with a rule-free cost model, so
on a line where marks were reordered (nested quotes, for example) the swapped
marks aligned as an insertion plus a deletion and were never counted. That
understated the forward probability of the closing quote, which pushed it just
under the reliability bar, so the map converted the opening quote but not the
closing one.

Feed each frequent substitution back as a cheap rule and re-align, the same
bootstrap the character rules already use, iterating to a fixed point. The
closing-quote rule now clears the bar and converts in both directions, the
inner quote pair becomes reversible, and the previously missing closing inner
rule appears. Word-internal apostrophes stay protected by the existing 'both'
class, so only word-edge possessives misfire, which is rare and accepted.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/British2American.xlsx
+++ b/examples/British2American.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CharPairs'!$A$1:$J$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'WordPairs'!$A$1:$K$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Lexicon'!$A$1:$E$88</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'PunctPairs'!$A$1:$G$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'PunctPairs'!$A$1:$G$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>data\oeb-british.txt</t>
+          <t>data/oeb-british.txt</t>
         </is>
       </c>
     </row>
@@ -480,7 +480,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>data\oeb-american.txt</t>
+          <t>data/oeb-american.txt</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>examples\oeb-chars.csv</t>
+          <t>examples/oeb-chars.csv</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>examples\British2American.map</t>
+          <t>examples/British2American.map</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="25">
@@ -7411,7 +7411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7419,7 +7419,7 @@
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -7472,13 +7472,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2111</v>
+        <v>2154</v>
       </c>
       <c r="D2" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>0.979</v>
+        <v>0.999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7503,17 +7503,17 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1990</v>
+        <v>2055</v>
       </c>
       <c r="D3" t="n">
-        <v>0.948</v>
+        <v>0.979</v>
       </c>
       <c r="E3" t="n">
-        <v>0.967</v>
+        <v>0.999</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>bwd</t>
+          <t>both</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -7534,17 +7534,17 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>857</v>
+        <v>901</v>
       </c>
       <c r="D4" t="n">
-        <v>0.949</v>
+        <v>0.998</v>
       </c>
       <c r="E4" t="n">
-        <v>0.951</v>
+        <v>1</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>bwd</t>
+          <t>both</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -7565,120 +7565,27 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>833</v>
+        <v>897</v>
       </c>
       <c r="D5" t="n">
-        <v>0.926</v>
+        <v>0.997</v>
       </c>
       <c r="E5" t="n">
-        <v>0.884</v>
+        <v>0.952</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>unreliable</t>
+          <t>both</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>7141, 12723, 12758, 12758, 12862</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>‘</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>”</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>unreliable</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>24543</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>“</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>’</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>unreliable</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>24800</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>’</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>“</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>unreliable</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>26134</t>
+          <t>7141, 12723, 12758, 12758, 12806</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G8"/>
+  <autoFilter ref="A1:G5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>